<commit_message>
Bổ sung môn Ngữ văn (Tiếng Việt lớp 2) vào agent giáo viên và thời khóa biểu
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B5wLyTmgHWgweec8EwAuG3
</commit_message>
<xml_diff>
--- a/hoc-tap/thoi-khoa-bieu.xlsx
+++ b/hoc-tap/thoi-khoa-bieu.xlsx
@@ -614,52 +614,53 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Khoa học tự nhiên</t>
+          <t>Ngữ văn
+Đọc hiểu văn bản, làm thẻ ôn</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Ngữ văn
+Đọc hiểu văn bản ngoài SGK</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Thứ 5</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>19:00–19:30
+Tiếng Việt
+Đọc to, chính tả, soát lỗi</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Toán</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Toán
 1 bài giải 2 cách</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Thứ 5</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Thứ 6</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>19:00–19:30
 Toán
-Bài có lời văn – gạch chân dữ kiện</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Toán</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>Tiếng Anh
-Đọc hiểu, viết lại câu</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Thứ 6</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>19:00–19:30
-Toán
-Luyện tính cẩn thận, ôn cả tuần</t>
+Bài có lời văn, tính cẩn thận</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
@@ -670,34 +671,35 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
+          <t>Ngữ văn
+Lập dàn ý, viết đoạn nghị luận</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Thứ 7</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>19:00–19:30
+Tiếng Việt
+Đọc truyện, kể lại, viết 3–5 câu
++ 5' Tiếng Anh trò chơi</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
           <t>KHTN (tuần lẻ)
 Lịch sử – Địa lý (tuần chẵn)</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Thứ 7</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>19:00–19:30
-Tiếng Anh + TNXH
-Dạng trò chơi</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Lịch sử – Địa lý
-Sơ đồ tư duy</t>
-        </is>
-      </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Mini đề thi vào 10 TP.HCM – 25'
-Tuần lẻ Toán, tuần chẵn Anh</t>
+Xoay vòng Toán → Anh → Văn</t>
         </is>
       </c>
     </row>
@@ -710,20 +712,20 @@
       <c r="B9" s="7" t="inlineStr">
         <is>
           <t>19:00–19:30
-Thám tử tìm lỗi sai
+Toán: thám tử tìm lỗi sai
 Đếm ⭐ cả tuần</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Kiểm tra nhanh 15' trộn cả tuần
-+ 15' ôn thẻ từ vựng</t>
++ 15' Ngữ văn: viết đoạn ngắn</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Chữa đề thứ 7
-Lỗi "chưa hiểu" hay "nhầm"</t>
+          <t>Chữa đề thứ 7 (15')
++ Tiếng Anh đọc hiểu, viết lại câu (15')</t>
         </is>
       </c>
     </row>
@@ -758,7 +760,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>Đầu tháng 12/2026 chuyển sang ôn thi học kỳ I. Từ tháng 3/2027 nên tăng thời gian của Khủng Long lên 45–60'/ngày.</t>
+          <t>KHTN, Lịch sử – Địa lý của Khủng Long: học trên lớp, ở nhà ôn khi sắp kiểm tra. Đầu tháng 12/2026 chuyển sang ôn thi học kỳ I. Từ tháng 3/2027 nên tăng thời gian của Khủng Long lên 45–60'/ngày.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Heo Mập: tối thứ 2, 4 nghỉ hoặc học nhẹ sau 20h, dồn môn sang ngày khác
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B5wLyTmgHWgweec8EwAuG3
</commit_message>
<xml_diff>
--- a/hoc-tap/thoi-khoa-bieu.xlsx
+++ b/hoc-tap/thoi-khoa-bieu.xlsx
@@ -556,9 +556,9 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>17:30–18:00
-Tiếng Anh (nhẹ)
-Từ vựng, hát, nói câu ngắn</t>
+          <t>Đi học thêm
+Nghỉ – hoặc sau 20:00 (tùy chọn)
+15' Tiếng Anh nhẹ: nghe hát, ôn từ</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -607,9 +607,9 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>17:30–18:00
-Tự nhiên và Xã hội (nhẹ)
-Kể chuyện, quan sát quanh nhà</t>
+          <t>Đi học thêm
+Nghỉ – hoặc sau 20:00 (tùy chọn)
+15' đọc truyện / video TNXH</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -685,9 +685,8 @@
       <c r="B8" s="7" t="inlineStr">
         <is>
           <t>19:00–19:30
-Tiếng Việt
-Đọc truyện, kể lại, viết 3–5 câu
-+ 5' Tiếng Anh trò chơi</t>
+Tiếng Anh (15') + TNXH (15')
+Dạng trò chơi</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -712,8 +711,8 @@
       <c r="B9" s="7" t="inlineStr">
         <is>
           <t>19:00–19:30
-Toán: thám tử tìm lỗi sai
-Đếm ⭐ cả tuần</t>
+Tiếng Việt: đọc truyện, kể lại (15')
++ Toán: thám tử tìm lỗi sai, đếm ⭐ (15')</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -739,7 +738,7 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>🐷 Heo Mập: 5' tính nhẩm chậm – chắc → 20' bài chính → 5' kiểm tra lại bài + nhận ⭐. Thứ 2, 4 đi học thêm buổi tối nên học ở nhà lúc 17:30.</t>
+          <t>🐷 Heo Mập: 5' tính nhẩm chậm – chắc → 20' bài chính → 5' kiểm tra lại bài + nhận ⭐. Thứ 2, 4 đi học thêm: nghỉ, hoặc học nhẹ 15' sau 20:00 nếu bé còn sức.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Khủng Long: Khoa học tự nhiên cố định tối thứ 6
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B5wLyTmgHWgweec8EwAuG3
</commit_message>
<xml_diff>
--- a/hoc-tap/thoi-khoa-bieu.xlsx
+++ b/hoc-tap/thoi-khoa-bieu.xlsx
@@ -621,7 +621,8 @@
       <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Ngữ văn
-Đọc hiểu văn bản ngoài SGK</t>
+Tuần lẻ: đọc hiểu văn bản ngoài SGK
+Tuần chẵn: lập dàn ý, viết đoạn nghị luận</t>
         </is>
       </c>
     </row>
@@ -671,8 +672,8 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>Ngữ văn
-Lập dàn ý, viết đoạn nghị luận</t>
+          <t>Khoa học tự nhiên
+Hiểu bản chất, bài tập Lý/Hóa/Sinh</t>
         </is>
       </c>
     </row>
@@ -759,7 +760,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>Khủng Long: Khoa học tự nhiên ôn ở nhà khi sắp kiểm tra; không học Lịch sử – Địa lý ở nhà. Đầu tháng 12/2026 chuyển sang ôn thi học kỳ I. Từ tháng 3/2027 nên tăng thời gian của Khủng Long lên 45–60'/ngày.</t>
+          <t>Khủng Long: không học Lịch sử – Địa lý ở nhà. Đầu tháng 12/2026 chuyển sang ôn thi học kỳ I. Từ tháng 3/2027 nên tăng thời gian của Khủng Long lên 45–60'/ngày.</t>
         </is>
       </c>
     </row>

</xml_diff>